<commit_message>
Update data for non-tender and completed tenders for 2026
- Modified metadata for non-tender realization, updating last updated date and removing key fields.
- Updated non-tender realization data in Excel format.
- Adjusted completed tender data CSV format, changing column order and updating entries.
- Updated completed tender data in JSON format to reflect new structure and entries.
- Modified metadata for completed tenders, updating last updated date.
- Updated completed tender data in Excel format.
- Revised runbook to reflect the latest status and procedures for data updates.
- Added new CSV file for affirmation of procurement planning data as of August 19, 2026.
</commit_message>
<xml_diff>
--- a/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
+++ b/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
@@ -401,88 +401,88 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>psr_id</v>
+      </c>
+      <c r="B1" t="str">
+        <v>tahun_anggaran</v>
+      </c>
+      <c r="C1" t="str">
+        <v>nilai_kontrak</v>
+      </c>
+      <c r="D1" t="str">
+        <v>npwp_16_penyedia</v>
+      </c>
+      <c r="E1" t="str">
+        <v>nilai_negosiasi</v>
+      </c>
+      <c r="F1" t="str">
+        <v>provinsi</v>
+      </c>
+      <c r="G1" t="str">
+        <v>lokasi_pekerjaan</v>
+      </c>
+      <c r="H1" t="str">
+        <v>kd_rup_paket</v>
+      </c>
+      <c r="I1" t="str">
+        <v>pagu</v>
+      </c>
+      <c r="J1" t="str">
+        <v>kd_tender</v>
+      </c>
+      <c r="K1" t="str">
+        <v>kd_penyedia</v>
+      </c>
+      <c r="L1" t="str">
+        <v>tgl_pengumuman_tender</v>
+      </c>
+      <c r="M1" t="str">
         <v>nilai_pdn_kontrak</v>
       </c>
-      <c r="B1" t="str">
-        <v>kd_tender</v>
-      </c>
-      <c r="C1" t="str">
+      <c r="N1" t="str">
+        <v>kabkota</v>
+      </c>
+      <c r="O1" t="str">
+        <v>kd_lpse</v>
+      </c>
+      <c r="P1" t="str">
+        <v>kd_satker</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>hps</v>
+      </c>
+      <c r="R1" t="str">
+        <v>kd_paket</v>
+      </c>
+      <c r="S1" t="str">
+        <v>nilai_terkoreksi</v>
+      </c>
+      <c r="T1" t="str">
+        <v>kd_klpd</v>
+      </c>
+      <c r="U1" t="str">
+        <v>jenis_klpd</v>
+      </c>
+      <c r="V1" t="str">
+        <v>nilai_penawaran</v>
+      </c>
+      <c r="W1" t="str">
+        <v>nama_penyedia</v>
+      </c>
+      <c r="X1" t="str">
+        <v>nilai_umk_kontrak</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>nama_klpd</v>
+      </c>
+      <c r="Z1" t="str">
         <v>nama_satker</v>
       </c>
-      <c r="D1" t="str">
-        <v>provinsi</v>
-      </c>
-      <c r="E1" t="str">
-        <v>tahun_anggaran</v>
-      </c>
-      <c r="F1" t="str">
-        <v>kabkota</v>
-      </c>
-      <c r="G1" t="str">
-        <v>kd_klpd</v>
-      </c>
-      <c r="H1" t="str">
-        <v>npwp_16_penyedia</v>
-      </c>
-      <c r="I1" t="str">
-        <v>kd_satker</v>
-      </c>
-      <c r="J1" t="str">
-        <v>nilai_negosiasi</v>
-      </c>
-      <c r="K1" t="str">
-        <v>pagu</v>
-      </c>
-      <c r="L1" t="str">
-        <v>nilai_penawaran</v>
-      </c>
-      <c r="M1" t="str">
-        <v>nilai_umk_kontrak</v>
-      </c>
-      <c r="N1" t="str">
-        <v>psr_id</v>
-      </c>
-      <c r="O1" t="str">
-        <v>kd_rup_paket</v>
-      </c>
-      <c r="P1" t="str">
-        <v>kd_paket</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>kd_lpse</v>
-      </c>
-      <c r="R1" t="str">
-        <v>lokasi_pekerjaan</v>
-      </c>
-      <c r="S1" t="str">
-        <v>nama_klpd</v>
-      </c>
-      <c r="T1" t="str">
-        <v>hps</v>
-      </c>
-      <c r="U1" t="str">
-        <v>kd_penyedia</v>
-      </c>
-      <c r="V1" t="str">
-        <v>nama_penyedia</v>
-      </c>
-      <c r="W1" t="str">
+      <c r="AA1" t="str">
+        <v>tgl_penetapan_pemenang</v>
+      </c>
+      <c r="AB1" t="str">
         <v>npwp_penyedia</v>
-      </c>
-      <c r="X1" t="str">
-        <v>nilai_terkoreksi</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>tgl_penetapan_pemenang</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>tgl_pengumuman_tender</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>jenis_klpd</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>nilai_kontrak</v>
       </c>
       <c r="AC1" t="str">
         <v>last_update_ref</v>
@@ -490,226 +490,226 @@
     </row>
     <row r="2">
       <c r="B2">
+        <v>2026</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Kalimantan Utara</v>
+      </c>
+      <c r="G2" t="str">
+        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
+      </c>
+      <c r="H2" t="str">
+        <v>66390319</v>
+      </c>
+      <c r="I2">
+        <v>108024405000</v>
+      </c>
+      <c r="J2">
         <v>10157189000</v>
       </c>
-      <c r="C2" t="str">
+      <c r="L2" t="str">
+        <v>2026-07-29T00:00:00Z</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Bulungan (Kab.)</v>
+      </c>
+      <c r="O2">
+        <v>194</v>
+      </c>
+      <c r="P2" t="str">
+        <v>626131</v>
+      </c>
+      <c r="Q2">
+        <v>94577629145</v>
+      </c>
+      <c r="R2">
+        <v>10150225000</v>
+      </c>
+      <c r="T2" t="str">
+        <v>K34</v>
+      </c>
+      <c r="U2" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="Z2" t="str">
         <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
       </c>
-      <c r="D2" t="str">
-        <v>Kalimantan Utara</v>
-      </c>
-      <c r="E2">
-        <v>2026</v>
-      </c>
-      <c r="F2" t="str">
-        <v>Bulungan (Kab.)</v>
-      </c>
-      <c r="G2" t="str">
-        <v>K34</v>
-      </c>
-      <c r="I2" t="str">
-        <v>626131</v>
-      </c>
-      <c r="K2">
-        <v>108024405000</v>
-      </c>
-      <c r="O2" t="str">
-        <v>66390319</v>
-      </c>
-      <c r="P2">
-        <v>10150225000</v>
-      </c>
-      <c r="Q2">
-        <v>194</v>
-      </c>
-      <c r="R2" t="str">
-        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
-      </c>
-      <c r="S2" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="T2">
-        <v>94577629145</v>
-      </c>
-      <c r="Y2" t="str">
+      <c r="AA2" t="str">
         <v>2026-09-03T00:00:00Z</v>
       </c>
-      <c r="Z2" t="str">
-        <v>2026-07-29T00:00:00Z</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC2" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.HUp3KgHOoKslxwmw.dyydQzJpCL9A1UM6coKqEu_vHnlSyJvCVHx3PZKM-ts</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
       </c>
     </row>
     <row r="3">
       <c r="B3">
+        <v>2026</v>
+      </c>
+      <c r="F3" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="G3" t="str">
+        <v>Jl. Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="H3" t="str">
+        <v>67611590</v>
+      </c>
+      <c r="I3">
+        <v>400000000</v>
+      </c>
+      <c r="J3">
         <v>10159515000</v>
       </c>
-      <c r="C3" t="str">
+      <c r="L3" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="O3">
+        <v>194</v>
+      </c>
+      <c r="P3" t="str">
+        <v>452677</v>
+      </c>
+      <c r="Q3">
+        <v>294600000</v>
+      </c>
+      <c r="R3">
+        <v>10152339000</v>
+      </c>
+      <c r="T3" t="str">
+        <v>K34</v>
+      </c>
+      <c r="U3" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="Z3" t="str">
         <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
       </c>
-      <c r="D3" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="E3">
-        <v>2026</v>
-      </c>
-      <c r="F3" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="G3" t="str">
-        <v>K34</v>
-      </c>
-      <c r="I3" t="str">
-        <v>452677</v>
-      </c>
-      <c r="K3">
-        <v>400000000</v>
-      </c>
-      <c r="O3" t="str">
-        <v>67611590</v>
-      </c>
-      <c r="P3">
-        <v>10152339000</v>
-      </c>
-      <c r="Q3">
-        <v>194</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Jl. Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="S3" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="T3">
-        <v>294600000</v>
-      </c>
-      <c r="Y3" t="str">
+      <c r="AA3" t="str">
         <v>2026-09-17T00:00:00Z</v>
       </c>
-      <c r="Z3" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="AA3" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC3" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.HUp3KgHOoKslxwmw.dyydQzJpCL9A1UM6coKqEu_vHnlSyJvCVHx3PZKM-ts</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
       </c>
     </row>
     <row r="4">
       <c r="B4">
+        <v>2026</v>
+      </c>
+      <c r="F4" t="str">
+        <v>Maluku Utara</v>
+      </c>
+      <c r="G4" t="str">
+        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
+      </c>
+      <c r="H4" t="str">
+        <v>66390318</v>
+      </c>
+      <c r="I4">
+        <v>72311690000</v>
+      </c>
+      <c r="J4">
         <v>10158222000</v>
       </c>
-      <c r="C4" t="str">
+      <c r="L4" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Halmahera Selatan (Kab.)</v>
+      </c>
+      <c r="O4">
+        <v>194</v>
+      </c>
+      <c r="P4" t="str">
+        <v>626131</v>
+      </c>
+      <c r="Q4">
+        <v>72210016000</v>
+      </c>
+      <c r="R4">
+        <v>10151157000</v>
+      </c>
+      <c r="T4" t="str">
+        <v>K34</v>
+      </c>
+      <c r="U4" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="Z4" t="str">
         <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
       </c>
-      <c r="D4" t="str">
-        <v>Maluku Utara</v>
-      </c>
-      <c r="E4">
-        <v>2026</v>
-      </c>
-      <c r="F4" t="str">
-        <v>Halmahera Selatan (Kab.)</v>
-      </c>
-      <c r="G4" t="str">
-        <v>K34</v>
-      </c>
-      <c r="I4" t="str">
-        <v>626131</v>
-      </c>
-      <c r="K4">
-        <v>72311690000</v>
-      </c>
-      <c r="O4" t="str">
-        <v>66390318</v>
-      </c>
-      <c r="P4">
-        <v>10151157000</v>
-      </c>
-      <c r="Q4">
-        <v>194</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
-      </c>
-      <c r="S4" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="T4">
-        <v>72210016000</v>
-      </c>
-      <c r="Y4" t="str">
+      <c r="AA4" t="str">
         <v>2026-09-16T00:00:00Z</v>
       </c>
-      <c r="Z4" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="AA4" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC4" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.HUp3KgHOoKslxwmw.dyydQzJpCL9A1UM6coKqEu_vHnlSyJvCVHx3PZKM-ts</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
       </c>
     </row>
     <row r="5">
       <c r="B5">
+        <v>2026</v>
+      </c>
+      <c r="F5" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="G5" t="str">
+        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
+      </c>
+      <c r="H5" t="str">
+        <v>67429813</v>
+      </c>
+      <c r="I5">
+        <v>2300000000</v>
+      </c>
+      <c r="J5">
         <v>10151353000</v>
       </c>
-      <c r="C5" t="str">
+      <c r="L5" t="str">
+        <v>2026-07-22T00:00:00Z</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="O5">
+        <v>194</v>
+      </c>
+      <c r="P5" t="str">
+        <v>626132</v>
+      </c>
+      <c r="Q5">
+        <v>2299921875</v>
+      </c>
+      <c r="R5">
+        <v>10144772000</v>
+      </c>
+      <c r="T5" t="str">
+        <v>K34</v>
+      </c>
+      <c r="U5" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="Z5" t="str">
         <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
       </c>
-      <c r="D5" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="E5">
-        <v>2026</v>
-      </c>
-      <c r="F5" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="G5" t="str">
-        <v>K34</v>
-      </c>
-      <c r="I5" t="str">
-        <v>626132</v>
-      </c>
-      <c r="K5">
-        <v>2300000000</v>
-      </c>
-      <c r="O5" t="str">
-        <v>67429813</v>
-      </c>
-      <c r="P5">
-        <v>10144772000</v>
-      </c>
-      <c r="Q5">
-        <v>194</v>
-      </c>
-      <c r="R5" t="str">
-        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
-      </c>
-      <c r="S5" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="T5">
-        <v>2299921875</v>
-      </c>
-      <c r="Y5" t="str">
-        <v>2026-08-18T00:00:00Z</v>
-      </c>
-      <c r="Z5" t="str">
-        <v>2026-07-22T00:00:00Z</v>
-      </c>
       <c r="AA5" t="str">
-        <v>KEMENTERIAN</v>
+        <v>2026-08-21T00:00:00Z</v>
       </c>
       <c r="AC5" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.HUp3KgHOoKslxwmw.dyydQzJpCL9A1UM6coKqEu_vHnlSyJvCVHx3PZKM-ts</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
Update Supabase data 20 Agustus 2026 dan tambah kolom hps
Tarikan data terbaru untuk 10 tabel via update_from_data_update.mjs.
Field baru `hps` di sumber pencatatan_non_tender_realisasi butuh
migration ALTER TABLE (68) sebelum bisa ditulis; database.types.ts
diregenerate mengikuti.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
+++ b/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
@@ -401,315 +401,315 @@
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>kabkota</v>
+      </c>
+      <c r="B1" t="str">
         <v>psr_id</v>
       </c>
-      <c r="B1" t="str">
+      <c r="C1" t="str">
+        <v>kd_satker</v>
+      </c>
+      <c r="D1" t="str">
+        <v>nilai_terkoreksi</v>
+      </c>
+      <c r="E1" t="str">
+        <v>npwp_penyedia</v>
+      </c>
+      <c r="F1" t="str">
+        <v>nilai_kontrak</v>
+      </c>
+      <c r="G1" t="str">
+        <v>nilai_penawaran</v>
+      </c>
+      <c r="H1" t="str">
+        <v>npwp_16_penyedia</v>
+      </c>
+      <c r="I1" t="str">
+        <v>tgl_pengumuman_tender</v>
+      </c>
+      <c r="J1" t="str">
+        <v>kd_lpse</v>
+      </c>
+      <c r="K1" t="str">
+        <v>nama_penyedia</v>
+      </c>
+      <c r="L1" t="str">
+        <v>nilai_pdn_kontrak</v>
+      </c>
+      <c r="M1" t="str">
+        <v>hps</v>
+      </c>
+      <c r="N1" t="str">
+        <v>tgl_penetapan_pemenang</v>
+      </c>
+      <c r="O1" t="str">
+        <v>kd_tender</v>
+      </c>
+      <c r="P1" t="str">
+        <v>kd_penyedia</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>nilai_umk_kontrak</v>
+      </c>
+      <c r="R1" t="str">
+        <v>nilai_negosiasi</v>
+      </c>
+      <c r="S1" t="str">
+        <v>kd_rup_paket</v>
+      </c>
+      <c r="T1" t="str">
+        <v>lokasi_pekerjaan</v>
+      </c>
+      <c r="U1" t="str">
+        <v>nama_klpd</v>
+      </c>
+      <c r="V1" t="str">
+        <v>kd_paket</v>
+      </c>
+      <c r="W1" t="str">
+        <v>kd_klpd</v>
+      </c>
+      <c r="X1" t="str">
+        <v>pagu</v>
+      </c>
+      <c r="Y1" t="str">
+        <v>nama_satker</v>
+      </c>
+      <c r="Z1" t="str">
+        <v>provinsi</v>
+      </c>
+      <c r="AA1" t="str">
         <v>tahun_anggaran</v>
       </c>
-      <c r="C1" t="str">
-        <v>nilai_kontrak</v>
-      </c>
-      <c r="D1" t="str">
-        <v>npwp_16_penyedia</v>
-      </c>
-      <c r="E1" t="str">
-        <v>nilai_negosiasi</v>
-      </c>
-      <c r="F1" t="str">
-        <v>provinsi</v>
-      </c>
-      <c r="G1" t="str">
-        <v>lokasi_pekerjaan</v>
-      </c>
-      <c r="H1" t="str">
-        <v>kd_rup_paket</v>
-      </c>
-      <c r="I1" t="str">
-        <v>pagu</v>
-      </c>
-      <c r="J1" t="str">
-        <v>kd_tender</v>
-      </c>
-      <c r="K1" t="str">
-        <v>kd_penyedia</v>
-      </c>
-      <c r="L1" t="str">
-        <v>tgl_pengumuman_tender</v>
-      </c>
-      <c r="M1" t="str">
-        <v>nilai_pdn_kontrak</v>
-      </c>
-      <c r="N1" t="str">
-        <v>kabkota</v>
-      </c>
-      <c r="O1" t="str">
-        <v>kd_lpse</v>
-      </c>
-      <c r="P1" t="str">
-        <v>kd_satker</v>
-      </c>
-      <c r="Q1" t="str">
-        <v>hps</v>
-      </c>
-      <c r="R1" t="str">
-        <v>kd_paket</v>
-      </c>
-      <c r="S1" t="str">
-        <v>nilai_terkoreksi</v>
-      </c>
-      <c r="T1" t="str">
-        <v>kd_klpd</v>
-      </c>
-      <c r="U1" t="str">
+      <c r="AB1" t="str">
         <v>jenis_klpd</v>
-      </c>
-      <c r="V1" t="str">
-        <v>nilai_penawaran</v>
-      </c>
-      <c r="W1" t="str">
-        <v>nama_penyedia</v>
-      </c>
-      <c r="X1" t="str">
-        <v>nilai_umk_kontrak</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>nama_klpd</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>nama_satker</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>tgl_penetapan_pemenang</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>npwp_penyedia</v>
       </c>
       <c r="AC1" t="str">
         <v>last_update_ref</v>
       </c>
     </row>
     <row r="2">
-      <c r="B2">
+      <c r="A2" t="str">
+        <v>Bulungan (Kab.)</v>
+      </c>
+      <c r="C2" t="str">
+        <v>626131</v>
+      </c>
+      <c r="I2" t="str">
+        <v>2026-07-29T00:00:00Z</v>
+      </c>
+      <c r="J2">
+        <v>194</v>
+      </c>
+      <c r="M2">
+        <v>94577629145</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2026-09-17T00:00:00Z</v>
+      </c>
+      <c r="O2">
+        <v>10157189000</v>
+      </c>
+      <c r="S2" t="str">
+        <v>66390319</v>
+      </c>
+      <c r="T2" t="str">
+        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
+      </c>
+      <c r="U2" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="V2">
+        <v>10150225000</v>
+      </c>
+      <c r="W2" t="str">
+        <v>K34</v>
+      </c>
+      <c r="X2">
+        <v>108024405000</v>
+      </c>
+      <c r="Y2" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="Z2" t="str">
+        <v>Kalimantan Utara</v>
+      </c>
+      <c r="AA2">
         <v>2026</v>
       </c>
-      <c r="F2" t="str">
-        <v>Kalimantan Utara</v>
-      </c>
-      <c r="G2" t="str">
-        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
-      </c>
-      <c r="H2" t="str">
-        <v>66390319</v>
-      </c>
-      <c r="I2">
-        <v>108024405000</v>
-      </c>
-      <c r="J2">
-        <v>10157189000</v>
-      </c>
-      <c r="L2" t="str">
-        <v>2026-07-29T00:00:00Z</v>
-      </c>
-      <c r="N2" t="str">
-        <v>Bulungan (Kab.)</v>
-      </c>
-      <c r="O2">
-        <v>194</v>
-      </c>
-      <c r="P2" t="str">
-        <v>626131</v>
-      </c>
-      <c r="Q2">
-        <v>94577629145</v>
-      </c>
-      <c r="R2">
-        <v>10150225000</v>
-      </c>
-      <c r="T2" t="str">
-        <v>K34</v>
-      </c>
-      <c r="U2" t="str">
+      <c r="AB2" t="str">
         <v>KEMENTERIAN</v>
       </c>
-      <c r="Y2" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="AA2" t="str">
-        <v>2026-09-03T00:00:00Z</v>
-      </c>
       <c r="AC2" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3">
+      <c r="A3" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="C3" t="str">
+        <v>452677</v>
+      </c>
+      <c r="I3" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="J3">
+        <v>194</v>
+      </c>
+      <c r="M3">
+        <v>294600000</v>
+      </c>
+      <c r="N3" t="str">
+        <v>2026-09-17T00:00:00Z</v>
+      </c>
+      <c r="O3">
+        <v>10159515000</v>
+      </c>
+      <c r="S3" t="str">
+        <v>67611590</v>
+      </c>
+      <c r="T3" t="str">
+        <v>Jl. Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="U3" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="V3">
+        <v>10152339000</v>
+      </c>
+      <c r="W3" t="str">
+        <v>K34</v>
+      </c>
+      <c r="X3">
+        <v>400000000</v>
+      </c>
+      <c r="Y3" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="Z3" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="AA3">
         <v>2026</v>
       </c>
-      <c r="F3" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="G3" t="str">
-        <v>Jl. Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="H3" t="str">
-        <v>67611590</v>
-      </c>
-      <c r="I3">
-        <v>400000000</v>
-      </c>
-      <c r="J3">
-        <v>10159515000</v>
-      </c>
-      <c r="L3" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="N3" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="O3">
-        <v>194</v>
-      </c>
-      <c r="P3" t="str">
-        <v>452677</v>
-      </c>
-      <c r="Q3">
-        <v>294600000</v>
-      </c>
-      <c r="R3">
-        <v>10152339000</v>
-      </c>
-      <c r="T3" t="str">
-        <v>K34</v>
-      </c>
-      <c r="U3" t="str">
+      <c r="AB3" t="str">
         <v>KEMENTERIAN</v>
       </c>
-      <c r="Y3" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="Z3" t="str">
-        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
-      </c>
-      <c r="AA3" t="str">
-        <v>2026-09-17T00:00:00Z</v>
-      </c>
       <c r="AC3" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4">
+      <c r="A4" t="str">
+        <v>Halmahera Selatan (Kab.)</v>
+      </c>
+      <c r="C4" t="str">
+        <v>626131</v>
+      </c>
+      <c r="I4" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="J4">
+        <v>194</v>
+      </c>
+      <c r="M4">
+        <v>72210016000</v>
+      </c>
+      <c r="N4" t="str">
+        <v>2026-09-16T00:00:00Z</v>
+      </c>
+      <c r="O4">
+        <v>10158222000</v>
+      </c>
+      <c r="S4" t="str">
+        <v>66390318</v>
+      </c>
+      <c r="T4" t="str">
+        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
+      </c>
+      <c r="U4" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="V4">
+        <v>10151157000</v>
+      </c>
+      <c r="W4" t="str">
+        <v>K34</v>
+      </c>
+      <c r="X4">
+        <v>72311690000</v>
+      </c>
+      <c r="Y4" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="Z4" t="str">
+        <v>Maluku Utara</v>
+      </c>
+      <c r="AA4">
         <v>2026</v>
       </c>
-      <c r="F4" t="str">
-        <v>Maluku Utara</v>
-      </c>
-      <c r="G4" t="str">
-        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
-      </c>
-      <c r="H4" t="str">
-        <v>66390318</v>
-      </c>
-      <c r="I4">
-        <v>72311690000</v>
-      </c>
-      <c r="J4">
-        <v>10158222000</v>
-      </c>
-      <c r="L4" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="N4" t="str">
-        <v>Halmahera Selatan (Kab.)</v>
-      </c>
-      <c r="O4">
-        <v>194</v>
-      </c>
-      <c r="P4" t="str">
-        <v>626131</v>
-      </c>
-      <c r="Q4">
-        <v>72210016000</v>
-      </c>
-      <c r="R4">
-        <v>10151157000</v>
-      </c>
-      <c r="T4" t="str">
-        <v>K34</v>
-      </c>
-      <c r="U4" t="str">
+      <c r="AB4" t="str">
         <v>KEMENTERIAN</v>
       </c>
-      <c r="Y4" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="Z4" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="AA4" t="str">
-        <v>2026-09-16T00:00:00Z</v>
-      </c>
       <c r="AC4" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5">
+      <c r="A5" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="C5" t="str">
+        <v>626132</v>
+      </c>
+      <c r="I5" t="str">
+        <v>2026-07-22T00:00:00Z</v>
+      </c>
+      <c r="J5">
+        <v>194</v>
+      </c>
+      <c r="M5">
+        <v>2299921875</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-08-21T00:00:00Z</v>
+      </c>
+      <c r="O5">
+        <v>10151353000</v>
+      </c>
+      <c r="S5" t="str">
+        <v>67429813</v>
+      </c>
+      <c r="T5" t="str">
+        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
+      </c>
+      <c r="U5" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="V5">
+        <v>10144772000</v>
+      </c>
+      <c r="W5" t="str">
+        <v>K34</v>
+      </c>
+      <c r="X5">
+        <v>2300000000</v>
+      </c>
+      <c r="Y5" t="str">
+        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
+      </c>
+      <c r="Z5" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="AA5">
         <v>2026</v>
       </c>
-      <c r="F5" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="G5" t="str">
-        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
-      </c>
-      <c r="H5" t="str">
-        <v>67429813</v>
-      </c>
-      <c r="I5">
-        <v>2300000000</v>
-      </c>
-      <c r="J5">
-        <v>10151353000</v>
-      </c>
-      <c r="L5" t="str">
-        <v>2026-07-22T00:00:00Z</v>
-      </c>
-      <c r="N5" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="O5">
-        <v>194</v>
-      </c>
-      <c r="P5" t="str">
-        <v>626132</v>
-      </c>
-      <c r="Q5">
-        <v>2299921875</v>
-      </c>
-      <c r="R5">
-        <v>10144772000</v>
-      </c>
-      <c r="T5" t="str">
-        <v>K34</v>
-      </c>
-      <c r="U5" t="str">
+      <c r="AB5" t="str">
         <v>KEMENTERIAN</v>
       </c>
-      <c r="Y5" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="Z5" t="str">
-        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
-      </c>
-      <c r="AA5" t="str">
-        <v>2026-08-21T00:00:00Z</v>
-      </c>
       <c r="AC5" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.K1igx_n_1BGp5LJ7.S1BdIdzPDVbI_5BoRwTAjlUZo0eq2lEwLzmuesfpV_Y</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
docs: add comprehensive documentation for DEWA-PBJ development journey across four phases
</commit_message>
<xml_diff>
--- a/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
+++ b/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
@@ -397,89 +397,89 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC5"/>
+  <dimension ref="A1:AC8"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
+        <v>nilai_umk_kontrak</v>
+      </c>
+      <c r="B1" t="str">
+        <v>tgl_pengumuman_tender</v>
+      </c>
+      <c r="C1" t="str">
+        <v>kd_rup_paket</v>
+      </c>
+      <c r="D1" t="str">
+        <v>hps</v>
+      </c>
+      <c r="E1" t="str">
+        <v>kd_klpd</v>
+      </c>
+      <c r="F1" t="str">
+        <v>provinsi</v>
+      </c>
+      <c r="G1" t="str">
+        <v>nilai_kontrak</v>
+      </c>
+      <c r="H1" t="str">
+        <v>kd_tender</v>
+      </c>
+      <c r="I1" t="str">
+        <v>nilai_negosiasi</v>
+      </c>
+      <c r="J1" t="str">
         <v>kabkota</v>
       </c>
-      <c r="B1" t="str">
-        <v>psr_id</v>
-      </c>
-      <c r="C1" t="str">
-        <v>kd_satker</v>
-      </c>
-      <c r="D1" t="str">
-        <v>nilai_terkoreksi</v>
-      </c>
-      <c r="E1" t="str">
-        <v>npwp_penyedia</v>
-      </c>
-      <c r="F1" t="str">
-        <v>nilai_kontrak</v>
-      </c>
-      <c r="G1" t="str">
+      <c r="K1" t="str">
+        <v>nama_klpd</v>
+      </c>
+      <c r="L1" t="str">
         <v>nilai_penawaran</v>
       </c>
-      <c r="H1" t="str">
-        <v>npwp_16_penyedia</v>
-      </c>
-      <c r="I1" t="str">
-        <v>tgl_pengumuman_tender</v>
-      </c>
-      <c r="J1" t="str">
-        <v>kd_lpse</v>
-      </c>
-      <c r="K1" t="str">
-        <v>nama_penyedia</v>
-      </c>
-      <c r="L1" t="str">
-        <v>nilai_pdn_kontrak</v>
-      </c>
       <c r="M1" t="str">
-        <v>hps</v>
+        <v>kd_paket</v>
       </c>
       <c r="N1" t="str">
         <v>tgl_penetapan_pemenang</v>
       </c>
       <c r="O1" t="str">
-        <v>kd_tender</v>
+        <v>lokasi_pekerjaan</v>
       </c>
       <c r="P1" t="str">
+        <v>tahun_anggaran</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>psr_id</v>
+      </c>
+      <c r="R1" t="str">
+        <v>nama_satker</v>
+      </c>
+      <c r="S1" t="str">
+        <v>nilai_terkoreksi</v>
+      </c>
+      <c r="T1" t="str">
+        <v>kd_satker</v>
+      </c>
+      <c r="U1" t="str">
         <v>kd_penyedia</v>
       </c>
-      <c r="Q1" t="str">
-        <v>nilai_umk_kontrak</v>
-      </c>
-      <c r="R1" t="str">
-        <v>nilai_negosiasi</v>
-      </c>
-      <c r="S1" t="str">
-        <v>kd_rup_paket</v>
-      </c>
-      <c r="T1" t="str">
-        <v>lokasi_pekerjaan</v>
-      </c>
-      <c r="U1" t="str">
-        <v>nama_klpd</v>
-      </c>
       <c r="V1" t="str">
-        <v>kd_paket</v>
+        <v>nama_penyedia</v>
       </c>
       <c r="W1" t="str">
-        <v>kd_klpd</v>
+        <v>nilai_pdn_kontrak</v>
       </c>
       <c r="X1" t="str">
+        <v>npwp_16_penyedia</v>
+      </c>
+      <c r="Y1" t="str">
         <v>pagu</v>
       </c>
-      <c r="Y1" t="str">
-        <v>nama_satker</v>
-      </c>
       <c r="Z1" t="str">
-        <v>provinsi</v>
+        <v>npwp_penyedia</v>
       </c>
       <c r="AA1" t="str">
-        <v>tahun_anggaran</v>
+        <v>kd_lpse</v>
       </c>
       <c r="AB1" t="str">
         <v>jenis_klpd</v>
@@ -489,232 +489,400 @@
       </c>
     </row>
     <row r="2">
-      <c r="A2" t="str">
-        <v>Bulungan (Kab.)</v>
+      <c r="B2" t="str">
+        <v>2026-08-21T00:00:00Z</v>
       </c>
       <c r="C2" t="str">
+        <v>66390312</v>
+      </c>
+      <c r="D2">
+        <v>51439625000</v>
+      </c>
+      <c r="E2" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F2" t="str">
+        <v>Bengkulu</v>
+      </c>
+      <c r="H2">
+        <v>10159959000</v>
+      </c>
+      <c r="J2" t="str">
+        <v>Bengkulu (Kota)</v>
+      </c>
+      <c r="K2" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M2">
+        <v>10152741000</v>
+      </c>
+      <c r="N2" t="str">
+        <v>2026-10-01T00:00:00Z</v>
+      </c>
+      <c r="O2" t="str">
+        <v>Jalan Merapi Raya No. 89, Kelurahan Panorama, Kecamatan Singaran Pati, Kota Bengkulu, Provinsi Bengkulu</v>
+      </c>
+      <c r="P2">
+        <v>2026</v>
+      </c>
+      <c r="R2" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="T2" t="str">
         <v>626131</v>
       </c>
-      <c r="I2" t="str">
-        <v>2026-07-29T00:00:00Z</v>
-      </c>
-      <c r="J2">
+      <c r="Y2">
+        <v>63441052000</v>
+      </c>
+      <c r="AA2">
         <v>194</v>
-      </c>
-      <c r="M2">
-        <v>94577629145</v>
-      </c>
-      <c r="N2" t="str">
-        <v>2026-09-17T00:00:00Z</v>
-      </c>
-      <c r="O2">
-        <v>10157189000</v>
-      </c>
-      <c r="S2" t="str">
-        <v>66390319</v>
-      </c>
-      <c r="T2" t="str">
-        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
-      </c>
-      <c r="U2" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="V2">
-        <v>10150225000</v>
-      </c>
-      <c r="W2" t="str">
-        <v>K34</v>
-      </c>
-      <c r="X2">
-        <v>108024405000</v>
-      </c>
-      <c r="Y2" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="Z2" t="str">
-        <v>Kalimantan Utara</v>
-      </c>
-      <c r="AA2">
-        <v>2026</v>
       </c>
       <c r="AB2" t="str">
         <v>KEMENTERIAN</v>
       </c>
       <c r="AC2" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
       </c>
     </row>
     <row r="3">
-      <c r="A3" t="str">
-        <v>Jakarta Selatan (Kota)</v>
+      <c r="B3" t="str">
+        <v>2026-07-29T00:00:00Z</v>
       </c>
       <c r="C3" t="str">
-        <v>452677</v>
-      </c>
-      <c r="I3" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="J3">
-        <v>194</v>
+        <v>66390319</v>
+      </c>
+      <c r="D3">
+        <v>94577629145</v>
+      </c>
+      <c r="E3" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F3" t="str">
+        <v>Kalimantan Utara</v>
+      </c>
+      <c r="H3">
+        <v>10157189000</v>
+      </c>
+      <c r="J3" t="str">
+        <v>Bulungan (Kab.)</v>
+      </c>
+      <c r="K3" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
       </c>
       <c r="M3">
-        <v>294600000</v>
+        <v>10150225000</v>
       </c>
       <c r="N3" t="str">
         <v>2026-09-17T00:00:00Z</v>
       </c>
-      <c r="O3">
-        <v>10159515000</v>
-      </c>
-      <c r="S3" t="str">
-        <v>67611590</v>
+      <c r="O3" t="str">
+        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
+      </c>
+      <c r="P3">
+        <v>2026</v>
+      </c>
+      <c r="R3" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
       </c>
       <c r="T3" t="str">
-        <v>Jl. Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="U3" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="V3">
-        <v>10152339000</v>
-      </c>
-      <c r="W3" t="str">
-        <v>K34</v>
-      </c>
-      <c r="X3">
-        <v>400000000</v>
-      </c>
-      <c r="Y3" t="str">
-        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
-      </c>
-      <c r="Z3" t="str">
-        <v>DKI Jakarta</v>
+        <v>626131</v>
+      </c>
+      <c r="Y3">
+        <v>108024405000</v>
       </c>
       <c r="AA3">
-        <v>2026</v>
+        <v>194</v>
       </c>
       <c r="AB3" t="str">
         <v>KEMENTERIAN</v>
       </c>
       <c r="AC3" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
       </c>
     </row>
     <row r="4">
-      <c r="A4" t="str">
-        <v>Halmahera Selatan (Kab.)</v>
+      <c r="B4" t="str">
+        <v>2026-08-05T00:00:00Z</v>
       </c>
       <c r="C4" t="str">
-        <v>626131</v>
-      </c>
-      <c r="I4" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="J4">
+        <v>67611590</v>
+      </c>
+      <c r="D4">
+        <v>294600000</v>
+      </c>
+      <c r="E4" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F4" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="H4">
+        <v>10159515000</v>
+      </c>
+      <c r="J4" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="K4" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M4">
+        <v>10152339000</v>
+      </c>
+      <c r="N4" t="str">
+        <v>2026-09-17T00:00:00Z</v>
+      </c>
+      <c r="O4" t="str">
+        <v>Jl. Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="P4">
+        <v>2026</v>
+      </c>
+      <c r="R4" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="T4" t="str">
+        <v>452677</v>
+      </c>
+      <c r="Y4">
+        <v>400000000</v>
+      </c>
+      <c r="AA4">
         <v>194</v>
-      </c>
-      <c r="M4">
-        <v>72210016000</v>
-      </c>
-      <c r="N4" t="str">
-        <v>2026-09-16T00:00:00Z</v>
-      </c>
-      <c r="O4">
-        <v>10158222000</v>
-      </c>
-      <c r="S4" t="str">
-        <v>66390318</v>
-      </c>
-      <c r="T4" t="str">
-        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
-      </c>
-      <c r="U4" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="V4">
-        <v>10151157000</v>
-      </c>
-      <c r="W4" t="str">
-        <v>K34</v>
-      </c>
-      <c r="X4">
-        <v>72311690000</v>
-      </c>
-      <c r="Y4" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="Z4" t="str">
-        <v>Maluku Utara</v>
-      </c>
-      <c r="AA4">
-        <v>2026</v>
       </c>
       <c r="AB4" t="str">
         <v>KEMENTERIAN</v>
       </c>
       <c r="AC4" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
       </c>
     </row>
     <row r="5">
-      <c r="A5" t="str">
+      <c r="B5" t="str">
+        <v>2026-08-21T00:00:00Z</v>
+      </c>
+      <c r="C5" t="str">
+        <v>67592003</v>
+      </c>
+      <c r="D5">
+        <v>12677050659</v>
+      </c>
+      <c r="E5" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F5" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="H5">
+        <v>10160960000</v>
+      </c>
+      <c r="J5" t="str">
         <v>Jakarta Selatan (Kota)</v>
       </c>
-      <c r="C5" t="str">
-        <v>626132</v>
-      </c>
-      <c r="I5" t="str">
-        <v>2026-07-22T00:00:00Z</v>
-      </c>
-      <c r="J5">
+      <c r="K5" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M5">
+        <v>10153666000</v>
+      </c>
+      <c r="N5" t="str">
+        <v>2026-10-07T00:00:00Z</v>
+      </c>
+      <c r="O5" t="str">
+        <v>Jl Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="P5">
+        <v>2026</v>
+      </c>
+      <c r="R5" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="T5" t="str">
+        <v>452677</v>
+      </c>
+      <c r="Y5">
+        <v>14699105000</v>
+      </c>
+      <c r="AA5">
         <v>194</v>
-      </c>
-      <c r="M5">
-        <v>2299921875</v>
-      </c>
-      <c r="N5" t="str">
-        <v>2026-08-21T00:00:00Z</v>
-      </c>
-      <c r="O5">
-        <v>10151353000</v>
-      </c>
-      <c r="S5" t="str">
-        <v>67429813</v>
-      </c>
-      <c r="T5" t="str">
-        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
-      </c>
-      <c r="U5" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="V5">
-        <v>10144772000</v>
-      </c>
-      <c r="W5" t="str">
-        <v>K34</v>
-      </c>
-      <c r="X5">
-        <v>2300000000</v>
-      </c>
-      <c r="Y5" t="str">
-        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
-      </c>
-      <c r="Z5" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="AA5">
-        <v>2026</v>
       </c>
       <c r="AB5" t="str">
         <v>KEMENTERIAN</v>
       </c>
       <c r="AC5" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.spw790JVkqpZ2DP_.Olrpwj3_aqYcd8ljKPV4RNIEDuUlJUlZ030Y3vHDOY0</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="B6" t="str">
+        <v>2026-08-20T00:00:00Z</v>
+      </c>
+      <c r="C6" t="str">
+        <v>67538462</v>
+      </c>
+      <c r="D6">
+        <v>646650000</v>
+      </c>
+      <c r="E6" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F6" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="H6">
+        <v>10162858000</v>
+      </c>
+      <c r="J6" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="K6" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M6">
+        <v>10155417000</v>
+      </c>
+      <c r="N6" t="str">
+        <v>2026-09-23T00:00:00Z</v>
+      </c>
+      <c r="O6" t="str">
+        <v>Jl Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="P6">
+        <v>2026</v>
+      </c>
+      <c r="R6" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="T6" t="str">
+        <v>452677</v>
+      </c>
+      <c r="Y6">
+        <v>654750000</v>
+      </c>
+      <c r="AA6">
+        <v>194</v>
+      </c>
+      <c r="AB6" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="AC6" t="str">
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="B7" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="C7" t="str">
+        <v>66390318</v>
+      </c>
+      <c r="D7">
+        <v>72210016000</v>
+      </c>
+      <c r="E7" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F7" t="str">
+        <v>Maluku Utara</v>
+      </c>
+      <c r="H7">
+        <v>10158222000</v>
+      </c>
+      <c r="J7" t="str">
+        <v>Halmahera Selatan (Kab.)</v>
+      </c>
+      <c r="K7" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M7">
+        <v>10151157000</v>
+      </c>
+      <c r="N7" t="str">
+        <v>2026-09-16T00:00:00Z</v>
+      </c>
+      <c r="O7" t="str">
+        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
+      </c>
+      <c r="P7">
+        <v>2026</v>
+      </c>
+      <c r="R7" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="T7" t="str">
+        <v>626131</v>
+      </c>
+      <c r="Y7">
+        <v>72311690000</v>
+      </c>
+      <c r="AA7">
+        <v>194</v>
+      </c>
+      <c r="AB7" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="AC7" t="str">
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="B8" t="str">
+        <v>2026-07-22T00:00:00Z</v>
+      </c>
+      <c r="C8" t="str">
+        <v>67429813</v>
+      </c>
+      <c r="D8">
+        <v>2299921875</v>
+      </c>
+      <c r="E8" t="str">
+        <v>K34</v>
+      </c>
+      <c r="F8" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="H8">
+        <v>10151353000</v>
+      </c>
+      <c r="J8" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="K8" t="str">
+        <v>Kementerian Ketenagakerjaan</v>
+      </c>
+      <c r="M8">
+        <v>10144772000</v>
+      </c>
+      <c r="N8" t="str">
+        <v>2026-08-26T00:00:00Z</v>
+      </c>
+      <c r="O8" t="str">
+        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
+      </c>
+      <c r="P8">
+        <v>2026</v>
+      </c>
+      <c r="R8" t="str">
+        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
+      </c>
+      <c r="T8" t="str">
+        <v>626132</v>
+      </c>
+      <c r="Y8">
+        <v>2300000000</v>
+      </c>
+      <c r="AA8">
+        <v>194</v>
+      </c>
+      <c r="AB8" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="AC8" t="str">
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC5"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC8"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>

<commit_message>
Update data files for tender and non-tender records for 2026
- Modified the structure of `tender-selesai-nilai_2026.csv` to reorder columns and update data entries.
- Updated `tender-selesai-nilai_2026.json` to reflect changes in the CSV structure and data.
- Adjusted metadata in `tender-selesai-nilai_2026.meta.json` to correct row count and last updated timestamp.
- Added new CSV file `data_afirmasi_pdn_perencanaan_20260826_021258.csv` containing procurement planning data.
- Updated binary files for `pencatatan-non-tender-realisasi_2026.xlsx` and `tender-selesai-nilai_2026.xlsx` to include new data.
</commit_message>
<xml_diff>
--- a/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
+++ b/data/data_update/tender_selesai_nilai/tender-selesai-nilai_2026.xlsx
@@ -397,492 +397,436 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:AC8"/>
+  <dimension ref="A1:AC7"/>
   <sheetData>
     <row r="1">
       <c r="A1" t="str">
-        <v>nilai_umk_kontrak</v>
+        <v>nama_penyedia</v>
       </c>
       <c r="B1" t="str">
-        <v>tgl_pengumuman_tender</v>
+        <v>kd_paket</v>
       </c>
       <c r="C1" t="str">
-        <v>kd_rup_paket</v>
+        <v>nilai_kontrak</v>
       </c>
       <c r="D1" t="str">
         <v>hps</v>
       </c>
       <c r="E1" t="str">
-        <v>kd_klpd</v>
+        <v>tgl_pengumuman_tender</v>
       </c>
       <c r="F1" t="str">
         <v>provinsi</v>
       </c>
       <c r="G1" t="str">
-        <v>nilai_kontrak</v>
+        <v>npwp_penyedia</v>
       </c>
       <c r="H1" t="str">
+        <v>nama_satker</v>
+      </c>
+      <c r="I1" t="str">
+        <v>pagu</v>
+      </c>
+      <c r="J1" t="str">
+        <v>kd_rup_paket</v>
+      </c>
+      <c r="K1" t="str">
+        <v>tahun_anggaran</v>
+      </c>
+      <c r="L1" t="str">
+        <v>kd_klpd</v>
+      </c>
+      <c r="M1" t="str">
+        <v>nilai_umk_kontrak</v>
+      </c>
+      <c r="N1" t="str">
+        <v>kabkota</v>
+      </c>
+      <c r="O1" t="str">
         <v>kd_tender</v>
       </c>
-      <c r="I1" t="str">
+      <c r="P1" t="str">
+        <v>lokasi_pekerjaan</v>
+      </c>
+      <c r="Q1" t="str">
+        <v>kd_lpse</v>
+      </c>
+      <c r="R1" t="str">
+        <v>nilai_pdn_kontrak</v>
+      </c>
+      <c r="S1" t="str">
+        <v>npwp_16_penyedia</v>
+      </c>
+      <c r="T1" t="str">
+        <v>jenis_klpd</v>
+      </c>
+      <c r="U1" t="str">
+        <v>kd_satker</v>
+      </c>
+      <c r="V1" t="str">
+        <v>nama_klpd</v>
+      </c>
+      <c r="W1" t="str">
+        <v>tgl_penetapan_pemenang</v>
+      </c>
+      <c r="X1" t="str">
+        <v>kd_penyedia</v>
+      </c>
+      <c r="Y1" t="str">
         <v>nilai_negosiasi</v>
       </c>
-      <c r="J1" t="str">
-        <v>kabkota</v>
-      </c>
-      <c r="K1" t="str">
-        <v>nama_klpd</v>
-      </c>
-      <c r="L1" t="str">
+      <c r="Z1" t="str">
+        <v>nilai_terkoreksi</v>
+      </c>
+      <c r="AA1" t="str">
         <v>nilai_penawaran</v>
       </c>
-      <c r="M1" t="str">
-        <v>kd_paket</v>
-      </c>
-      <c r="N1" t="str">
-        <v>tgl_penetapan_pemenang</v>
-      </c>
-      <c r="O1" t="str">
-        <v>lokasi_pekerjaan</v>
-      </c>
-      <c r="P1" t="str">
-        <v>tahun_anggaran</v>
-      </c>
-      <c r="Q1" t="str">
+      <c r="AB1" t="str">
         <v>psr_id</v>
-      </c>
-      <c r="R1" t="str">
-        <v>nama_satker</v>
-      </c>
-      <c r="S1" t="str">
-        <v>nilai_terkoreksi</v>
-      </c>
-      <c r="T1" t="str">
-        <v>kd_satker</v>
-      </c>
-      <c r="U1" t="str">
-        <v>kd_penyedia</v>
-      </c>
-      <c r="V1" t="str">
-        <v>nama_penyedia</v>
-      </c>
-      <c r="W1" t="str">
-        <v>nilai_pdn_kontrak</v>
-      </c>
-      <c r="X1" t="str">
-        <v>npwp_16_penyedia</v>
-      </c>
-      <c r="Y1" t="str">
-        <v>pagu</v>
-      </c>
-      <c r="Z1" t="str">
-        <v>npwp_penyedia</v>
-      </c>
-      <c r="AA1" t="str">
-        <v>kd_lpse</v>
-      </c>
-      <c r="AB1" t="str">
-        <v>jenis_klpd</v>
       </c>
       <c r="AC1" t="str">
         <v>last_update_ref</v>
       </c>
     </row>
     <row r="2">
-      <c r="B2" t="str">
-        <v>2026-08-21T00:00:00Z</v>
-      </c>
-      <c r="C2" t="str">
-        <v>66390312</v>
+      <c r="B2">
+        <v>10152741000</v>
       </c>
       <c r="D2">
         <v>51439625000</v>
       </c>
       <c r="E2" t="str">
-        <v>K34</v>
+        <v>2026-08-21T00:00:00Z</v>
       </c>
       <c r="F2" t="str">
         <v>Bengkulu</v>
       </c>
-      <c r="H2">
+      <c r="H2" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="I2">
+        <v>63441052000</v>
+      </c>
+      <c r="J2" t="str">
+        <v>66390312</v>
+      </c>
+      <c r="K2">
+        <v>2026</v>
+      </c>
+      <c r="L2" t="str">
+        <v>K34</v>
+      </c>
+      <c r="N2" t="str">
+        <v>Bengkulu (Kota)</v>
+      </c>
+      <c r="O2">
         <v>10159959000</v>
       </c>
-      <c r="J2" t="str">
-        <v>Bengkulu (Kota)</v>
-      </c>
-      <c r="K2" t="str">
+      <c r="P2" t="str">
+        <v>Jalan Merapi Raya No. 89, Kelurahan Panorama, Kecamatan Singaran Pati, Kota Bengkulu, Provinsi Bengkulu</v>
+      </c>
+      <c r="Q2">
+        <v>194</v>
+      </c>
+      <c r="T2" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U2" t="str">
+        <v>626131</v>
+      </c>
+      <c r="V2" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M2">
-        <v>10152741000</v>
-      </c>
-      <c r="N2" t="str">
+      <c r="W2" t="str">
         <v>2026-10-01T00:00:00Z</v>
       </c>
-      <c r="O2" t="str">
-        <v>Jalan Merapi Raya No. 89, Kelurahan Panorama, Kecamatan Singaran Pati, Kota Bengkulu, Provinsi Bengkulu</v>
-      </c>
-      <c r="P2">
-        <v>2026</v>
-      </c>
-      <c r="R2" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="T2" t="str">
-        <v>626131</v>
-      </c>
-      <c r="Y2">
-        <v>63441052000</v>
-      </c>
-      <c r="AA2">
-        <v>194</v>
-      </c>
-      <c r="AB2" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC2" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
     <row r="3">
-      <c r="B3" t="str">
-        <v>2026-07-29T00:00:00Z</v>
-      </c>
-      <c r="C3" t="str">
-        <v>66390319</v>
+      <c r="B3">
+        <v>10150225000</v>
       </c>
       <c r="D3">
         <v>94577629145</v>
       </c>
       <c r="E3" t="str">
-        <v>K34</v>
+        <v>2026-07-29T00:00:00Z</v>
       </c>
       <c r="F3" t="str">
         <v>Kalimantan Utara</v>
       </c>
-      <c r="H3">
+      <c r="H3" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="I3">
+        <v>108024405000</v>
+      </c>
+      <c r="J3" t="str">
+        <v>66390319</v>
+      </c>
+      <c r="K3">
+        <v>2026</v>
+      </c>
+      <c r="L3" t="str">
+        <v>K34</v>
+      </c>
+      <c r="N3" t="str">
+        <v>Bulungan (Kab.)</v>
+      </c>
+      <c r="O3">
         <v>10157189000</v>
       </c>
-      <c r="J3" t="str">
-        <v>Bulungan (Kab.)</v>
-      </c>
-      <c r="K3" t="str">
+      <c r="P3" t="str">
+        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
+      </c>
+      <c r="Q3">
+        <v>194</v>
+      </c>
+      <c r="T3" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U3" t="str">
+        <v>626131</v>
+      </c>
+      <c r="V3" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M3">
-        <v>10150225000</v>
-      </c>
-      <c r="N3" t="str">
+      <c r="W3" t="str">
         <v>2026-09-17T00:00:00Z</v>
       </c>
-      <c r="O3" t="str">
-        <v>Jalan Nasional Poros Bulungan - Malinau, Desa Seriang, Kecamatan Tanjung Selor, Kabupaten Bulungan, Provinsi Kalimantan Utara</v>
-      </c>
-      <c r="P3">
-        <v>2026</v>
-      </c>
-      <c r="R3" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="T3" t="str">
-        <v>626131</v>
-      </c>
-      <c r="Y3">
-        <v>108024405000</v>
-      </c>
-      <c r="AA3">
-        <v>194</v>
-      </c>
-      <c r="AB3" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC3" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
     <row r="4">
-      <c r="B4" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="C4" t="str">
-        <v>67611590</v>
+      <c r="B4">
+        <v>10152339000</v>
       </c>
       <c r="D4">
         <v>294600000</v>
       </c>
       <c r="E4" t="str">
-        <v>K34</v>
+        <v>2026-08-05T00:00:00Z</v>
       </c>
       <c r="F4" t="str">
         <v>DKI Jakarta</v>
       </c>
-      <c r="H4">
+      <c r="H4" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="I4">
+        <v>400000000</v>
+      </c>
+      <c r="J4" t="str">
+        <v>67611590</v>
+      </c>
+      <c r="K4">
+        <v>2026</v>
+      </c>
+      <c r="L4" t="str">
+        <v>K34</v>
+      </c>
+      <c r="N4" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="O4">
         <v>10159515000</v>
       </c>
-      <c r="J4" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="K4" t="str">
+      <c r="P4" t="str">
+        <v>Jl. Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="Q4">
+        <v>194</v>
+      </c>
+      <c r="T4" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U4" t="str">
+        <v>452677</v>
+      </c>
+      <c r="V4" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M4">
-        <v>10152339000</v>
-      </c>
-      <c r="N4" t="str">
+      <c r="W4" t="str">
         <v>2026-09-17T00:00:00Z</v>
       </c>
-      <c r="O4" t="str">
-        <v>Jl. Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="P4">
-        <v>2026</v>
-      </c>
-      <c r="R4" t="str">
-        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
-      </c>
-      <c r="T4" t="str">
-        <v>452677</v>
-      </c>
-      <c r="Y4">
-        <v>400000000</v>
-      </c>
-      <c r="AA4">
-        <v>194</v>
-      </c>
-      <c r="AB4" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC4" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
     <row r="5">
-      <c r="B5" t="str">
-        <v>2026-08-21T00:00:00Z</v>
-      </c>
-      <c r="C5" t="str">
-        <v>67592003</v>
+      <c r="B5">
+        <v>10153666000</v>
       </c>
       <c r="D5">
         <v>12677050659</v>
       </c>
       <c r="E5" t="str">
-        <v>K34</v>
+        <v>2026-08-21T00:00:00Z</v>
       </c>
       <c r="F5" t="str">
         <v>DKI Jakarta</v>
       </c>
-      <c r="H5">
+      <c r="H5" t="str">
+        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
+      </c>
+      <c r="I5">
+        <v>14699105000</v>
+      </c>
+      <c r="J5" t="str">
+        <v>67592003</v>
+      </c>
+      <c r="K5">
+        <v>2026</v>
+      </c>
+      <c r="L5" t="str">
+        <v>K34</v>
+      </c>
+      <c r="N5" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="O5">
         <v>10160960000</v>
       </c>
-      <c r="J5" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="K5" t="str">
+      <c r="P5" t="str">
+        <v>Jl Jend Gatot Subroto Kav 51</v>
+      </c>
+      <c r="Q5">
+        <v>194</v>
+      </c>
+      <c r="T5" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U5" t="str">
+        <v>452677</v>
+      </c>
+      <c r="V5" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M5">
-        <v>10153666000</v>
-      </c>
-      <c r="N5" t="str">
+      <c r="W5" t="str">
         <v>2026-10-07T00:00:00Z</v>
       </c>
-      <c r="O5" t="str">
-        <v>Jl Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="P5">
-        <v>2026</v>
-      </c>
-      <c r="R5" t="str">
-        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
-      </c>
-      <c r="T5" t="str">
-        <v>452677</v>
-      </c>
-      <c r="Y5">
-        <v>14699105000</v>
-      </c>
-      <c r="AA5">
-        <v>194</v>
-      </c>
-      <c r="AB5" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
       <c r="AC5" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
     <row r="6">
-      <c r="B6" t="str">
-        <v>2026-08-20T00:00:00Z</v>
-      </c>
-      <c r="C6" t="str">
-        <v>67538462</v>
+      <c r="B6">
+        <v>10151157000</v>
       </c>
       <c r="D6">
-        <v>646650000</v>
+        <v>72210016000</v>
       </c>
       <c r="E6" t="str">
+        <v>2026-08-05T00:00:00Z</v>
+      </c>
+      <c r="F6" t="str">
+        <v>Maluku Utara</v>
+      </c>
+      <c r="H6" t="str">
+        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
+      </c>
+      <c r="I6">
+        <v>72311690000</v>
+      </c>
+      <c r="J6" t="str">
+        <v>66390318</v>
+      </c>
+      <c r="K6">
+        <v>2026</v>
+      </c>
+      <c r="L6" t="str">
         <v>K34</v>
       </c>
-      <c r="F6" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="H6">
-        <v>10162858000</v>
-      </c>
-      <c r="J6" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="K6" t="str">
+      <c r="N6" t="str">
+        <v>Halmahera Selatan (Kab.)</v>
+      </c>
+      <c r="O6">
+        <v>10158222000</v>
+      </c>
+      <c r="P6" t="str">
+        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
+      </c>
+      <c r="Q6">
+        <v>194</v>
+      </c>
+      <c r="T6" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U6" t="str">
+        <v>626131</v>
+      </c>
+      <c r="V6" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M6">
-        <v>10155417000</v>
-      </c>
-      <c r="N6" t="str">
-        <v>2026-09-23T00:00:00Z</v>
-      </c>
-      <c r="O6" t="str">
-        <v>Jl Jend Gatot Subroto Kav 51</v>
-      </c>
-      <c r="P6">
-        <v>2026</v>
-      </c>
-      <c r="R6" t="str">
-        <v>Badan Perencanaan dan Pengembangan Ketenagakerjaan</v>
-      </c>
-      <c r="T6" t="str">
-        <v>452677</v>
-      </c>
-      <c r="Y6">
-        <v>654750000</v>
-      </c>
-      <c r="AA6">
-        <v>194</v>
-      </c>
-      <c r="AB6" t="str">
-        <v>KEMENTERIAN</v>
+      <c r="W6" t="str">
+        <v>2026-09-16T00:00:00Z</v>
       </c>
       <c r="AC6" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
     <row r="7">
-      <c r="B7" t="str">
-        <v>2026-08-05T00:00:00Z</v>
-      </c>
-      <c r="C7" t="str">
-        <v>66390318</v>
+      <c r="B7">
+        <v>10144772000</v>
       </c>
       <c r="D7">
-        <v>72210016000</v>
+        <v>2299921875</v>
       </c>
       <c r="E7" t="str">
+        <v>2026-07-22T00:00:00Z</v>
+      </c>
+      <c r="F7" t="str">
+        <v>DKI Jakarta</v>
+      </c>
+      <c r="H7" t="str">
+        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
+      </c>
+      <c r="I7">
+        <v>2300000000</v>
+      </c>
+      <c r="J7" t="str">
+        <v>67429813</v>
+      </c>
+      <c r="K7">
+        <v>2026</v>
+      </c>
+      <c r="L7" t="str">
         <v>K34</v>
       </c>
-      <c r="F7" t="str">
-        <v>Maluku Utara</v>
-      </c>
-      <c r="H7">
-        <v>10158222000</v>
-      </c>
-      <c r="J7" t="str">
-        <v>Halmahera Selatan (Kab.)</v>
-      </c>
-      <c r="K7" t="str">
+      <c r="N7" t="str">
+        <v>Jakarta Selatan (Kota)</v>
+      </c>
+      <c r="O7">
+        <v>10151353000</v>
+      </c>
+      <c r="P7" t="str">
+        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
+      </c>
+      <c r="Q7">
+        <v>194</v>
+      </c>
+      <c r="T7" t="str">
+        <v>KEMENTERIAN</v>
+      </c>
+      <c r="U7" t="str">
+        <v>626132</v>
+      </c>
+      <c r="V7" t="str">
         <v>Kementerian Ketenagakerjaan</v>
       </c>
-      <c r="M7">
-        <v>10151157000</v>
-      </c>
-      <c r="N7" t="str">
-        <v>2026-09-16T00:00:00Z</v>
-      </c>
-      <c r="O7" t="str">
-        <v>Desa Panamboang, Kecamatan Bacan Selatan, Kabupaten Halmahera Selatan, Provinsi Maluku Utara</v>
-      </c>
-      <c r="P7">
-        <v>2026</v>
-      </c>
-      <c r="R7" t="str">
-        <v>Direktorat Bina Kelembagaan Pelatihan Vokasi</v>
-      </c>
-      <c r="T7" t="str">
-        <v>626131</v>
-      </c>
-      <c r="Y7">
-        <v>72311690000</v>
-      </c>
-      <c r="AA7">
-        <v>194</v>
-      </c>
-      <c r="AB7" t="str">
-        <v>KEMENTERIAN</v>
+      <c r="W7" t="str">
+        <v>2026-08-26T00:00:00Z</v>
       </c>
       <c r="AC7" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
-      </c>
-    </row>
-    <row r="8">
-      <c r="B8" t="str">
-        <v>2026-07-22T00:00:00Z</v>
-      </c>
-      <c r="C8" t="str">
-        <v>67429813</v>
-      </c>
-      <c r="D8">
-        <v>2299921875</v>
-      </c>
-      <c r="E8" t="str">
-        <v>K34</v>
-      </c>
-      <c r="F8" t="str">
-        <v>DKI Jakarta</v>
-      </c>
-      <c r="H8">
-        <v>10151353000</v>
-      </c>
-      <c r="J8" t="str">
-        <v>Jakarta Selatan (Kota)</v>
-      </c>
-      <c r="K8" t="str">
-        <v>Kementerian Ketenagakerjaan</v>
-      </c>
-      <c r="M8">
-        <v>10144772000</v>
-      </c>
-      <c r="N8" t="str">
-        <v>2026-08-26T00:00:00Z</v>
-      </c>
-      <c r="O8" t="str">
-        <v>Gedung Vokasi Jalan Jenderal Gatot Subroto Kaveling 44 Jakarta Selatan DKI Jakarta</v>
-      </c>
-      <c r="P8">
-        <v>2026</v>
-      </c>
-      <c r="R8" t="str">
-        <v>Direktorat Bina Penyelenggaraan Pelatihan Vokasi dan Pemagangan</v>
-      </c>
-      <c r="T8" t="str">
-        <v>626132</v>
-      </c>
-      <c r="Y8">
-        <v>2300000000</v>
-      </c>
-      <c r="AA8">
-        <v>194</v>
-      </c>
-      <c r="AB8" t="str">
-        <v>KEMENTERIAN</v>
-      </c>
-      <c r="AC8" t="str">
-        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.cfGQhqjeisnhEK0l.olftb-mSmY5rQCNxtVl09-PYPC4Of48sJfJcus4O92w</v>
+        <v>cc820c5f-e6ba-5337-bc51-523cc40dc3a2.p0ZzV3QVc-16QjBE.0yNacvEeYvJ9--dFvzWKvXFxcr680TtcS9Z7azM4J0Q</v>
       </c>
     </row>
   </sheetData>
   <ignoredErrors>
-    <ignoredError numberStoredAsText="1" sqref="A1:AC8"/>
+    <ignoredError numberStoredAsText="1" sqref="A1:AC7"/>
   </ignoredErrors>
 </worksheet>
 </file>
</xml_diff>